<commit_message>
feat: ajustes modulo prestamo devolucion y merma
</commit_message>
<xml_diff>
--- a/Custom/AS_NSP_018_PrestamoDevolucionMerma/documentacion/excel/Casos_Negocio_AS_NSP_018_PrestamoDevolucionMerma.xlsx
+++ b/Custom/AS_NSP_018_PrestamoDevolucionMerma/documentacion/excel/Casos_Negocio_AS_NSP_018_PrestamoDevolucionMerma.xlsx
@@ -34,13 +34,11 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -67,16 +65,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00BFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00BFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00BFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00BFBFBF"/>
       </bottom>
     </border>
   </borders>
@@ -89,10 +87,10 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -459,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -502,7 +500,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="112" customHeight="1">
+    <row r="2" ht="102" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>0.1</t>
@@ -534,7 +532,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="112" customHeight="1">
+    <row r="3" ht="88" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>0.2</t>
@@ -561,6 +559,38 @@
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Víctor Raúl Huaman Simeon</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="144" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Devolución; Préstamo A la Clínica; comprobante; menú de configuración</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Mejora</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>En la devolución, si el lote del préstamo ya no tiene en la bodega de préstamos todo lo que se devuelve, el sistema completa la cantidad con otros lotes del mismo artículo y solo rechaza la devolución si entre todos no alcanza; cada línea muestra los lotes devueltos con su cantidad. En el préstamo A la Clínica el lote pasa a ser obligatorio en todas las líneas. El comprobante de préstamo y de devolución muestra el sentido del préstamo. Las opciones del menú de configuración pasan a llamarse Entidades Asociadas por Subsidiaria y Cuentas por Tipo de Movimiento.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Víctor Raúl Huaman Simeon</t>
         </is>
@@ -577,7 +607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -644,7 +674,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="70" customHeight="1">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>RN-001</t>
@@ -693,7 +723,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>RN-002</t>
@@ -741,7 +771,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="60" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>RN-003</t>
@@ -764,7 +794,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>El sistema muestra en Entidad Receptora del Prestamo solo las entidades activas cargadas para la subsidiaria en Entidades Receptoras.</t>
+          <t>El sistema muestra en Entidad Receptora del Prestamo solo las entidades activas cargadas para la subsidiaria en Entidades Asociadas por Subsidiaria.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -774,22 +804,26 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr"/>
+          <t>Modificada</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>La opción del menú se llama Entidades Asociadas por Subsidiaria</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1">
+          <t>22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>RN-004</t>
@@ -837,7 +871,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
+    <row r="6" ht="32" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>RN-005</t>
@@ -885,7 +919,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="98" customHeight="1">
+    <row r="7" ht="88" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>RN-046</t>
@@ -909,7 +943,7 @@
       <c r="E7" s="2" t="inlineStr">
         <is>
           <t>El sistema recarga el formulario: el grupo pasa a llamarse «2. Destino», no muestra Ubicacion Origen, la entidad pasa a llamarse Entidad Emisora del Prestamo y pide Cuenta de Ajuste como obligatoria.
-En los artículos, Lote se escribe a mano y no se muestra Disponible.</t>
+En los artículos, Lote se escribe a mano y es obligatorio, y no se muestra Disponible.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -919,22 +953,26 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr"/>
+          <t>Modificada</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>El lote pasa a ser obligatorio en todas las líneas</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="56" customHeight="1">
+          <t>22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>RN-047</t>
@@ -957,7 +995,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>El sistema muestra en Cuenta de Ajuste solo las cuentas activas de la subsidiaria cargadas en Cuentas de Merma con Tipo de Solicitud Prestamo.</t>
+          <t>El sistema muestra en Cuenta de Ajuste solo las cuentas activas de la subsidiaria cargadas en Cuentas por Tipo de Movimiento con Tipo de Solicitud Prestamo.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -967,22 +1005,26 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr"/>
+          <t>Modificada</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>La opción del menú se llama Cuentas por Tipo de Movimiento</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="56" customHeight="1">
+          <t>22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="74" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>RN-048</t>
@@ -995,7 +1037,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Préstamo A la Clínica con un artículo con control de lotes en el que no se escribió lote, al presionar Guardar Solicitud</t>
+          <t>Préstamo A la Clínica: agregar un artículo sin escribir el lote</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1005,32 +1047,36 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>El sistema muestra «Indica un lote para los articulos con control de lotes en las lineas [n].» y no guarda.</t>
+          <t>El sistema no acepta la línea y pide completar Lote, que es obligatorio en todas las líneas del préstamo A la Clínica, tenga o no el artículo control de lotes.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Préstamo no guardado</t>
+          <t>Línea no agregada</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
+          <t>Modificada</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>El formulario exige el lote en todas las líneas, al agregarlas y no recién al guardar</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="84" customHeight="1">
+          <t>22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="74" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>RN-054</t>
@@ -1079,7 +1125,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
+    <row r="11" ht="32" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>RN-006</t>
@@ -1127,7 +1173,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="84" customHeight="1">
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>RN-007</t>
@@ -1176,7 +1222,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="42" customHeight="1">
+    <row r="13" ht="32" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>RN-008</t>
@@ -1224,7 +1270,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="42" customHeight="1">
+    <row r="14" ht="32" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>RN-009</t>
@@ -1272,7 +1318,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="42" customHeight="1">
+    <row r="15" ht="32" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>RN-010</t>
@@ -1320,7 +1366,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="56" customHeight="1">
+    <row r="16" ht="32" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>RN-011</t>
@@ -1368,7 +1414,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="42" customHeight="1">
+    <row r="17" ht="32" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>RN-012</t>
@@ -1416,7 +1462,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="42" customHeight="1">
+    <row r="18" ht="32" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>RN-013</t>
@@ -1464,7 +1510,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="70" customHeight="1">
+    <row r="19" ht="60" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>RN-014</t>
@@ -1513,7 +1559,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="56" customHeight="1">
+    <row r="20" ht="46" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>RN-015</t>
@@ -1561,7 +1607,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="42" customHeight="1">
+    <row r="21" ht="32" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t>RN-016</t>
@@ -1609,7 +1655,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="56" customHeight="1">
+    <row r="22" ht="46" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>RN-017</t>
@@ -1657,7 +1703,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="84" customHeight="1">
+    <row r="23" ht="74" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t>RN-049</t>
@@ -1706,7 +1752,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="84" customHeight="1">
+    <row r="24" ht="60" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
           <t>RN-018</t>
@@ -1758,7 +1804,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="98" customHeight="1">
+    <row r="25" ht="88" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
           <t>RN-019</t>
@@ -1807,7 +1853,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="112" customHeight="1">
+    <row r="26" ht="88" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
           <t>RN-020</t>
@@ -1856,7 +1902,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="56" customHeight="1">
+    <row r="27" ht="32" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
           <t>RN-050</t>
@@ -1904,7 +1950,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="84" customHeight="1">
+    <row r="28" ht="74" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
         <is>
           <t>RN-051</t>
@@ -1953,7 +1999,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="56" customHeight="1">
+    <row r="29" ht="32" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t>RN-021</t>
@@ -2001,7 +2047,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="42" customHeight="1">
+    <row r="30" ht="32" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
         <is>
           <t>RN-022</t>
@@ -2049,7 +2095,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="42" customHeight="1">
+    <row r="31" ht="32" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>RN-023</t>
@@ -2097,7 +2143,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="98" customHeight="1">
+    <row r="32" ht="74" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
         <is>
           <t>RN-024</t>
@@ -2146,7 +2192,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="56" customHeight="1">
+    <row r="33" ht="32" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
           <t>RN-025</t>
@@ -2194,7 +2240,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="70" customHeight="1">
+    <row r="34" ht="60" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
         <is>
           <t>RN-026</t>
@@ -2242,7 +2288,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="42" customHeight="1">
+    <row r="35" ht="32" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>RN-027</t>
@@ -2290,7 +2336,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="56" customHeight="1">
+    <row r="36" ht="46" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
         <is>
           <t>RN-028</t>
@@ -2338,7 +2384,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="56" customHeight="1">
+    <row r="37" ht="46" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
         <is>
           <t>RN-029</t>
@@ -2386,7 +2432,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="98" customHeight="1">
+    <row r="38" ht="88" customHeight="1">
       <c r="A38" s="3" t="inlineStr">
         <is>
           <t>RN-052</t>
@@ -2409,7 +2455,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>El sistema genera un ajuste de inventario que descuenta el material de la bodega de préstamos, con el lote del préstamo y contra la cuenta del préstamo, y muestra el lote en cada línea de la devolución.
+          <t>El sistema genera un ajuste de inventario que descuenta el material de la bodega de préstamos, con el lote del préstamo y contra la cuenta del préstamo, y muestra en cada línea de la devolución el lote devuelto con su cantidad.
 Descuenta lo devuelto en Devuelta y Pendiente del préstamo.</t>
         </is>
       </c>
@@ -2420,22 +2466,26 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr"/>
+          <t>Modificada</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>La línea muestra el lote con la cantidad devuelta, y si el lote no alcanza se completa con otros lotes</t>
+        </is>
+      </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="42" customHeight="1">
+          <t>22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="74" customHeight="1">
       <c r="A39" s="3" t="inlineStr">
         <is>
           <t>RN-053</t>
@@ -2448,7 +2498,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Procesar una devolución A la Clínica cuando en la bodega de préstamos ya no hay lo que se devuelve</t>
+          <t>Procesar una devolución cuando en la bodega de préstamos, sumando todos los lotes del artículo, no hay lo que se devuelve</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2458,65 +2508,70 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>El sistema muestra «No hay stock suficiente en [ubicación]: [artículo] lote [lote] (devuelve [N], hay [M])» y no genera el ajuste.</t>
+          <t>El sistema muestra «No hay stock suficiente en [ubicación]: [artículo] (devuelve [N], hay [M])» y no genera el traslado ni el ajuste.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Devolución en Pendiente de Procesar, sin ajuste</t>
+          <t>Devolución en Pendiente de Procesar, sin traslado ni ajuste</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="inlineStr"/>
+          <t>Modificada</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Aplica a los dos sentidos y solo cuando ningún otro lote del artículo cubre la diferencia</t>
+        </is>
+      </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="42" customHeight="1">
+          <t>22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="102" customHeight="1">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>RN-030</t>
+          <t>RN-055</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Registro de merma</t>
+          <t>Procesamiento de devolución</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Registrar una merma</t>
+          <t>Procesar una devolución cuando el lote del préstamo ya no tiene en la bodega de préstamos todo lo que se devuelve, pero otros lotes del mismo artículo sí</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>QF CASPM o Administrator</t>
+          <t>Sistema (automático)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>El sistema no muestra Ubicacion Destino ni Entidad Receptora, y pide Motivo de la Baja y Cuenta de Ajuste como obligatorios.</t>
+          <t>El sistema toma primero lo que queda del lote del préstamo y completa la diferencia con otros lotes del artículo en la bodega, en el mismo orden automático que usa cuando no se elige lote.
+Cada línea de la devolución muestra los lotes devueltos con su cantidad, por ejemplo «LOTE-A (3)» y «LOTE-B (2)», separados por una barra vertical.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Formulario de merma</t>
+          <t>Devolución en Procesado; préstamo en Devuelto Parcial o Devuelto Total</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2527,14 +2582,14 @@
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="28" customHeight="1">
+          <t>22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="32" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>RN-031</t>
+          <t>RN-030</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2544,7 +2599,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Merma sin motivo de baja</t>
+          <t>Registrar una merma</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2554,12 +2609,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>El sistema no guarda y pide completar Motivo de la Baja.</t>
+          <t>El sistema no muestra Ubicacion Destino ni Entidad Receptora, y pide Motivo de la Baja y Cuenta de Ajuste como obligatorios.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Merma no guardada</t>
+          <t>Formulario de merma</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -2579,10 +2634,10 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="42" customHeight="1">
+    <row r="42" ht="18" customHeight="1">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>RN-032</t>
+          <t>RN-031</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2592,7 +2647,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Merma en una subsidiaria con cuentas de merma activas e inactivas</t>
+          <t>Merma sin motivo de baja</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2602,12 +2657,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>El sistema muestra en Cuenta de Ajuste solo las cuentas activas cargadas para la subsidiaria en Cuentas de Merma.</t>
+          <t>El sistema no guarda y pide completar Motivo de la Baja.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Cuenta elegida de la lista autorizada</t>
+          <t>Merma no guardada</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -2627,283 +2682,287 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="42" customHeight="1">
+    <row r="43" ht="60" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
         <is>
+          <t>RN-032</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Registro de merma</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Merma en una subsidiaria con cuentas de merma activas e inactivas</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>QF CASPM o Administrator</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>El sistema muestra en Cuenta de Ajuste solo las cuentas activas cargadas para la subsidiaria en Cuentas por Tipo de Movimiento, con Tipo de Solicitud Merma o vacío.</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta elegida de la lista autorizada</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Modificada</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>La opción del menú se llama Cuentas por Tipo de Movimiento</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="32" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
           <t>RN-033</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Registro de merma</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Merma en una subsidiaria sin cuentas de merma activas</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>QF CASPM o Administrator</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>QF CASPM o Administrator</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>El sistema deja Cuenta de Ajuste vacía. Como es obligatoria, no deja guardar.</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Merma no guardada</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr"/>
-      <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="70" customHeight="1">
-      <c r="A44" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="60" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>RN-034</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>Procesamiento de merma</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>Procesar una merma con stock suficiente</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>QF CASPM o Administrator</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>QF CASPM o Administrator</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>El sistema genera un ajuste de inventario que descuenta el material de la misma ubicación, contra la cuenta elegida.
 Ajuste Generado muestra el ajuste.</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>Merma en Procesado, material fuera del inventario</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>Modificada</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr">
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t>El campo se llama Ajuste Generado en la merma, no Traslado Generado</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr">
+      <c r="J45" s="2" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="56" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
+    <row r="46" ht="46" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>RN-035</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Procesamiento de merma</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Dos mermas guardadas del mismo artículo y lote, cada una por todo lo que hay del lote: se procesa la primera y después la segunda</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>QF CASPM o Administrator</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>QF CASPM o Administrator</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>El sistema procesa la primera. En la segunda muestra «No hay stock suficiente en [ubicación]: [artículo] lote [lote] (da de baja [N], hay 0)» y no genera el ajuste.</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Segunda merma en Pendiente de Procesar, sin ajuste</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="inlineStr"/>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="98" customHeight="1">
-      <c r="A46" s="3" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="88" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>RN-036</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>Corrección y anulación</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Editar un préstamo o una merma en Pendiente de Procesar</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>QF CASPM o Administrator</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>QF CASPM o Administrator</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>El sistema abre la edición y guarda con Actualizar Solicitud los cambios de fecha, responsable, comentarios y artículos (en la merma y en el préstamo A la Clínica, también la cuenta de ajuste).
 Tipo, sentido (De la Clinica / A la Clinica), subsidiaria, servicio, ubicaciones, entidad y motivo aparecen bloqueados.</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>Solicitud corregida, sigue en Pendiente de Procesar</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>Modificada</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr">
         <is>
           <t>Se agregan el sentido y la cuenta del préstamo A la Clínica</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="J47" s="2" t="inlineStr">
         <is>
           <t>07/10/2026</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="98" customHeight="1">
-      <c r="A47" s="3" t="inlineStr">
+    <row r="48" ht="88" customHeight="1">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>RN-037</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>Corrección y anulación</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Editar una solicitud que ya no está en Pendiente de Procesar</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>QF CASPM o Administrator</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>QF CASPM o Administrator</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>El sistema no muestra el botón Editar en la solicitud.
 Si se usa Editar desde la lista, vuelve a la solicitud con el aviso «Este movimiento ya no se puede editar» y el texto «El movimiento esta en estado [estado]. Solo se puede editar mientras esta en Pendiente de Procesar.»</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>Solicitud sin cambios</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="I47" s="2" t="inlineStr"/>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="42" customHeight="1">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>RN-038</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Corrección y anulación</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Presionar Anular Movimiento en una solicitud Pendiente de Procesar y cancelar la confirmación</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>QF CASPM o Administrator</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>El sistema pregunta «Se anulara el movimiento. Confirma?» y, al cancelar, no hace nada.</t>
-        </is>
-      </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Solicitud sin cambios</t>
@@ -2926,10 +2985,10 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="56" customHeight="1">
+    <row r="49" ht="32" customHeight="1">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>RN-039</t>
+          <t>RN-038</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -2939,7 +2998,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Presionar Anular Movimiento en una solicitud Pendiente de Procesar y aceptar la confirmación</t>
+          <t>Presionar Anular Movimiento en una solicitud Pendiente de Procesar y cancelar la confirmación</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -2949,12 +3008,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>El sistema cambia el estado sin mover inventario y quita los botones de procesar, editar y anular. Se puede seguir consultando e imprimiendo.</t>
+          <t>El sistema pregunta «Se anulara el movimiento. Confirma?» y, al cancelar, no hace nada.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Solicitud en Anulado</t>
+          <t>Solicitud sin cambios</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -2974,35 +3033,35 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="42" customHeight="1">
+    <row r="50" ht="32" customHeight="1">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>RN-040</t>
+          <t>RN-039</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Consulta e impresión</t>
+          <t>Corrección y anulación</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Presionar Imprimir Comprobante en un préstamo, una devolución, una merma o una solicitud anulada</t>
+          <t>Presionar Anular Movimiento en una solicitud Pendiente de Procesar y aceptar la confirmación</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Cualquier rol</t>
+          <t>QF CASPM o Administrator</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>El sistema abre el comprobante en PDF con la plantilla del tipo de solicitud.</t>
+          <t>El sistema cambia el estado sin mover inventario y quita los botones de procesar, editar y anular. Se puede seguir consultando e imprimiendo.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Comprobante generado</t>
+          <t>Solicitud en Anulado</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -3022,83 +3081,88 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="42" customHeight="1">
+    <row r="51" ht="88" customHeight="1">
       <c r="A51" s="3" t="inlineStr">
         <is>
+          <t>RN-040</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Consulta e impresión</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Presionar Imprimir Comprobante en un préstamo, una devolución, una merma o una solicitud anulada</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Cualquier rol</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>El sistema abre el comprobante en PDF con la plantilla del tipo de solicitud.
+En el préstamo y la devolución muestra el sentido del préstamo. En el préstamo A la Clínica la entidad aparece como «Entidad emisora del prestamo» y no se muestra la ubicación de origen.</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Comprobante generado</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Modificada</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>El comprobante muestra el sentido del préstamo</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="32" customHeight="1">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
           <t>RN-041</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>Consulta e impresión</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>Abrir una solicitud con un rol distinto de QF CASPM y Administrator</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>Rol de consulta</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>El sistema muestra la solicitud sin el botón Editar, sin las opciones de eliminar y copiar, y sin botones de proceso ni de anulación.</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Solo lectura</t>
-        </is>
-      </c>
-      <c r="G51" s="2" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="I51" s="2" t="inlineStr"/>
-      <c r="J51" s="2" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="42" customHeight="1">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>RN-042</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>Consulta e impresión</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Crear una solicitud con un rol distinto de QF CASPM y Administrator</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>Rol de consulta</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>El sistema muestra la pantalla «Movimiento de Inventario - Solo Consulta» con el aviso «Tu rol es de solo consulta».</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>Solicitud no creada</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -3118,84 +3182,84 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="70" customHeight="1">
+    <row r="53" ht="32" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
         <is>
+          <t>RN-042</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Consulta e impresión</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Crear una solicitud con un rol distinto de QF CASPM y Administrator</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Rol de consulta</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>El sistema muestra la pantalla «Movimiento de Inventario - Solo Consulta» con el aviso «Tu rol es de solo consulta».</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Solicitud no creada</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="46" customHeight="1">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
           <t>RN-043</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>Configuración</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>Marcar como inactiva una entidad receptora que tiene un préstamo pendiente</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>Administrator</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>El sistema deja de ofrecer esa entidad al registrar préstamos.
 El préstamo pendiente de esa entidad sigue apareciendo para devolver.</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Entidad inactiva, préstamos ya hechos sin cambios</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="H53" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="I53" s="2" t="inlineStr"/>
-      <c r="J53" s="2" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="42" customHeight="1">
-      <c r="A54" s="3" t="inlineStr">
-        <is>
-          <t>RN-044</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>Configuración</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>Marcar como inactiva una cuenta de merma</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>Administrator</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>El sistema deja de ofrecer esa cuenta en Cuenta de Ajuste para esa subsidiaria.</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta inactiva</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -3215,50 +3279,98 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="84" customHeight="1">
+    <row r="55" ht="32" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
         <is>
+          <t>RN-044</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Configuración</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Marcar como inactiva una cuenta de merma</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Administrator</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>El sistema deja de ofrecer esa cuenta en Cuenta de Ajuste para esa subsidiaria.</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta inactiva</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="74" customHeight="1">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
           <t>RN-045</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Configuración</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Cambiar la bodega de préstamos de una subsidiaria a otra ubicación</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>Administrator</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>El sistema usa la bodega nueva como destino de los préstamos que se registren desde ese momento.
 Las devoluciones de préstamos ya procesados salen de la bodega que quedó guardada en cada préstamo.</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Cambio no retroactivo, préstamos previos sin modificación</t>
         </is>
       </c>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="H55" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="I55" s="2" t="inlineStr"/>
-      <c r="J55" s="2" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr">
         <is>
           <t>01/10/2026</t>
         </is>

</xml_diff>